<commit_message>
Aggiunge invio email promemoria scadenze (Gmail API) e deploy Railway
- Promemoria automatico scadenze taratura a 10gg via script schedulabile
- Invio email via Gmail API/OAuth2 (fallback SMTP), pulsante "Invia email ora" in dashboard
- Procfile/requirements.txt per deploy su Railway
</commit_message>
<xml_diff>
--- a/riparazionischede.xlsx
+++ b/riparazionischede.xlsx
@@ -579,7 +579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -631,313 +631,313 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2025-08-09</t>
+          <t>2025-01-21</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SCH-3007</t>
+          <t>SCH-3010</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Scheda monitoraggio temperatura motore trazione</t>
+          <t>Scheda regolatore climatizzazione</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>DTR-041</t>
+          <t>DTR0001</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Umidità infiltrata nel case</t>
+          <t>Componente bruciato per sovratensione</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Resistore di pull-up</t>
+          <t>Connettore antenna GPS</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Federica Galli</t>
+          <t>Marco Bianchi</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2025-08-20</t>
+          <t>2025-04-07</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>SCH-3002</t>
+          <t>SCH-3007</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Scheda driver freno elettropneumatico</t>
+          <t>Scheda monitoraggio temperatura motore trazione</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>TLS-102</t>
+          <t>S-2201</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Corto circuito su alimentazione</t>
+          <t>Interferenza elettromagnetica su sensore</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Fusibile di linea</t>
+          <t>Transceiver CAN</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Simone Ricci</t>
+          <t>Giulia Moretti</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2025-09-12</t>
+          <t>2025-04-20</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>SCH-3001</t>
+          <t>SCH-3005</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Scheda alimentatore ausiliario 24VCC</t>
+          <t>Scheda gateway comunicazione MVB/CAN</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>S-2214</t>
+          <t>TLS-102</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Componente bruciato per sovratensione</t>
+          <t>Ossidazione contatti</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Regolatore di tensione LM7805</t>
+          <t>Transistor di potenza MOSFET</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Luca Marino</t>
+          <t>Davide Colombo</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2025-09-28</t>
+          <t>2025-05-13</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>SCH-3005</t>
+          <t>SCH-3010</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Scheda gateway comunicazione MVB/CAN</t>
+          <t>Scheda regolatore climatizzazione</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>TLS-133</t>
+          <t>DTR-027</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Guasto su circuito di comunicazione</t>
+          <t>Sovraccarico termico componente di potenza</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Transceiver CAN</t>
+          <t>Diodo di protezione</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Elisa Bruno</t>
+          <t>Chiara Ferrari</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2025-10-14</t>
+          <t>2025-07-03</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>SCH-3004</t>
+          <t>SCH-3009</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Scheda encoder velocità assile</t>
+          <t>Scheda amplificatore segnale antenna GPS</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>TLS-118</t>
+          <t>DTR-014</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Interferenza elettromagnetica su sensore</t>
+          <t>Sovraccarico termico componente di potenza</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Sensore encoder ottico</t>
+          <t>Resistore di pull-up</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Luca Marino</t>
+          <t>Simone Ricci</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2025-11-05</t>
+          <t>2025-08-09</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>SCH-3003</t>
+          <t>SCH-3007</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Scheda interfaccia display cabina</t>
+          <t>Scheda monitoraggio temperatura motore trazione</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>DTR-014</t>
+          <t>DTR-041</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Saldatura a freddo su connettore</t>
+          <t>Umidità infiltrata nel case</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Connettore display</t>
+          <t>Resistore di pull-up</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Elisa Bruno</t>
+          <t>Federica Galli</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2025-11-27</t>
+          <t>2025-08-20</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>SCH-3009</t>
+          <t>SCH-3002</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Scheda amplificatore segnale antenna GPS</t>
+          <t>Scheda driver freno elettropneumatico</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>TLS-147</t>
+          <t>TLS-102</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Rottura meccanica connettore</t>
+          <t>Corto circuito su alimentazione</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Connettore antenna GPS</t>
+          <t>Fusibile di linea</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Luca Marino</t>
+          <t>Simone Ricci</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-08-29</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>SCH-3006</t>
+          <t>SCH-3005</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Scheda controllo porte automatiche</t>
+          <t>Scheda gateway comunicazione MVB/CAN</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>S-2255</t>
+          <t>TLS-118</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Rottura meccanica connettore</t>
+          <t>Saldatura a freddo su connettore</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Relè di potenza</t>
+          <t>Sensore encoder ottico</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Simone Ricci</t>
+          <t>Davide Colombo</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2025-09-12</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>SCH-3008</t>
+          <t>SCH-3001</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Scheda I/O digitale cabina</t>
+          <t>Scheda alimentatore ausiliario 24VCC</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -947,44 +947,44 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Corto circuito su alimentazione</t>
+          <t>Componente bruciato per sovratensione</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Diodo di protezione</t>
+          <t>Regolatore di tensione LM7805</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Elisa Bruno</t>
+          <t>Luca Marino</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2025-09-12</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>SCH-3004</t>
+          <t>SCH-3003</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Scheda encoder velocità assile</t>
+          <t>Scheda interfaccia display cabina</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>TLS-118</t>
+          <t>DTR0001</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Rottura meccanica connettore</t>
+          <t>Umidita' infiltrata nel case</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -994,88 +994,88 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Simone Ricci</t>
+          <t>Federica Galli</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2025-09-16</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>SCH-3001</t>
+          <t>SCH-3003</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Scheda alimentatore ausiliario 24VCC</t>
+          <t>Scheda interfaccia display cabina</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>S-2214</t>
+          <t>TLS-118</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Condensatore elettrolitico esaurito</t>
+          <t>Saldatura a freddo su connettore</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Condensatore elettrolitico 470uF</t>
+          <t>Regolatore di tensione LM7805</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Federica Galli</t>
+          <t>Luca Marino</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2025-09-28</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>SCH-3010</t>
+          <t>SCH-3005</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Scheda regolatore climatizzazione</t>
+          <t>Scheda gateway comunicazione MVB/CAN</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>S-2201</t>
+          <t>TLS-133</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Componente bruciato per sovratensione</t>
+          <t>Guasto su circuito di comunicazione</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Condensatore elettrolitico 470uF</t>
+          <t>Transceiver CAN</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Simone Ricci</t>
+          <t>Elisa Bruno</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2025-10-04</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1090,29 +1090,29 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>TLS-133</t>
+          <t>DTR-027</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Guasto su circuito di comunicazione</t>
+          <t>Rottura meccanica connettore</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Transceiver CAN</t>
+          <t>Connettore antenna GPS</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Luca Marino</t>
+          <t>Davide Colombo</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2025-10-14</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1142,44 +1142,1339 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Federica Galli</t>
+          <t>Luca Marino</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>2025-10-19</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3002</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Scheda driver freno elettropneumatico</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>TLS-102</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Condensatore elettrolitico esaurito</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Condensatore elettrolitico 470uF</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Simone Ricci</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-01</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3009</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Scheda amplificatore segnale antenna GPS</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>DTR-041</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Componente bruciato per sovratensione</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Condensatore elettrolitico 470uF</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Davide Colombo</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-03</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3006</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Scheda controllo porte automatiche</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>TLS-118</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Condensatore elettrolitico esaurito</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Connettore encoder</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Davide Colombo</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-04</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3006</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Scheda controllo porte automatiche</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>DTR-027</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Saldatura a freddo su connettore</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Connettore display</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Giulia Moretti</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-05</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3003</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Scheda interfaccia display cabina</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>DTR-014</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Saldatura a freddo su connettore</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Connettore display</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Elisa Bruno</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-27</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3009</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Scheda amplificatore segnale antenna GPS</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>TLS-147</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Rottura meccanica connettore</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Connettore antenna GPS</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Luca Marino</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3006</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Scheda controllo porte automatiche</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>S-2255</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Rottura meccanica connettore</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Relè di potenza</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Simone Ricci</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-13</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3005</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Scheda gateway comunicazione MVB/CAN</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>S-2201</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Rottura meccanica connettore</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Connettore display</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Marco Bianchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-24</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3008</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Scheda I/O digitale cabina</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>TLS-118</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Umidita' infiltrata nel case</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Connettore encoder</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Marco Bianchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3003</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Scheda interfaccia display cabina</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>TLS-133</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Interferenza elettromagnetica su sensore</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Rele' di potenza</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Elisa Bruno</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3007</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Scheda monitoraggio temperatura motore trazione</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>DTR-014</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Rottura meccanica connettore</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Optoisolatore</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Davide Colombo</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3008</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Scheda I/O digitale cabina</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>S-2214</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Corto circuito su alimentazione</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Diodo di protezione</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Elisa Bruno</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3004</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Scheda encoder velocità assile</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>TLS-118</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Rottura meccanica connettore</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Connettore encoder</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Simone Ricci</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3002</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Scheda driver freno elettropneumatico</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>TLS-118</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Guasto su circuito di comunicazione</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Rele' di potenza</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Giulia Moretti</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3001</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Scheda alimentatore ausiliario 24VCC</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>S-2214</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Condensatore elettrolitico esaurito</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Condensatore elettrolitico 470uF</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Federica Galli</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3004</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Scheda encoder velocità assile</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>S-2201</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Condensatore elettrolitico esaurito</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Transceiver CAN</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Luca Marino</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3006</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Scheda controllo porte automatiche</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>S-2201</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Umidita' infiltrata nel case</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Resistore di pull-up</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Marco Bianchi</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3010</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Scheda regolatore climatizzazione</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Dtr4</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Saldatura a freddo su connettore</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Fusibile di linea</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Simone Ricci</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3010</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Scheda regolatore climatizzazione</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>S-2201</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Componente bruciato per sovratensione</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Condensatore elettrolitico 470uF</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Simone Ricci</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3009</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Scheda amplificatore segnale antenna GPS</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>S-2201</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Rottura meccanica connettore</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Condensatore elettrolitico 470uF</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Elisa Bruno</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3005</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Scheda gateway comunicazione MVB/CAN</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>TLS-133</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Guasto su circuito di comunicazione</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Transceiver CAN</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Luca Marino</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3004</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Scheda encoder velocità assile</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>TLS-133</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Sovraccarico termico componente di potenza</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Connettore display</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Luca Marino</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3009</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Scheda amplificatore segnale antenna GPS</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>DTR-014</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Condensatore elettrolitico esaurito</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Transistor di potenza MOSFET</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Simone Ricci</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3001</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Scheda alimentatore ausiliario 24VCC</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>DTR-041</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Condensatore elettrolitico esaurito</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Resistore di pull-up</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Elisa Bruno</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3002</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Scheda driver freno elettropneumatico</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>DTR-041</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Componente bruciato per sovratensione</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Connettore antenna GPS</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Luca Marino</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3001</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Scheda alimentatore ausiliario 24VCC</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>S-2255</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Corto circuito su alimentazione</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Condensatore elettrolitico 470uF</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Federica Galli</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3004</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Scheda encoder velocità assile</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>TLS-118</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Interferenza elettromagnetica su sensore</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Sensore encoder ottico</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Federica Galli</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>SCH-3010</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>Scheda regolatore climatizzazione</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>S-2201</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>Componente bruciato per sovratensione</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>Condensatore elettrolitico 470uF</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr">
         <is>
           <t>Federica Galli</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3004</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Scheda encoder velocità assile</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>TLS-133</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Corto circuito su alimentazione</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Transceiver CAN</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Luca Marino</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3008</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Scheda I/O digitale cabina</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Dtr4</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Condensatore elettrolitico esaurito</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Regolatore di tensione LM7805</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Davide Colombo</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3006</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Scheda controllo porte automatiche</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>DTR-014</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Sovraccarico termico componente di potenza</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Rele' di potenza</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Simone Ricci</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3007</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Scheda monitoraggio temperatura motore trazione</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>TLS-102</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Interferenza elettromagnetica su sensore</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Connettore encoder</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Luca Marino</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3010</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Scheda regolatore climatizzazione</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>S-2201</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Condensatore elettrolitico esaurito</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Diodo di protezione</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Davide Colombo</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3009</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Scheda amplificatore segnale antenna GPS</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>S-2214</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Condensatore elettrolitico esaurito</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Sensore encoder ottico</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Simone Ricci</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3004</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Scheda encoder velocità assile</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>TLS-118</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Saldatura a freddo su connettore</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Transceiver CAN</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Chiara Ferrari</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>SCH-3005</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Scheda gateway comunicazione MVB/CAN</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>DTR-014</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Rottura meccanica connettore</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Optoisolatore</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Simone Ricci</t>
         </is>
       </c>
     </row>

</xml_diff>